<commit_message>
Version FunSearch 100/100 - Architecture complète
- 100/100 conjectures réfutées
- Temps total: 109 secondes
- Architecture FunSearch avec LLM
- Heuristique direction-aware
</commit_message>
<xml_diff>
--- a/results_counterexamples.xlsx
+++ b/results_counterexamples.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,393 +424,308 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>x</t>
+          <t>found</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>y</t>
+          <t>x_invariant</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>score</t>
+          <t>y_invariant</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>x_value</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>y_value</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>violation</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>nodes</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>edges</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>x_value</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>y_value</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>graph6</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>phase</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>evaluations</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>elapsed_s</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>886</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>maximum_degree</t>
-        </is>
+        <v>6466</v>
+      </c>
+      <c r="B2" t="b">
+        <v>1</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
           <t>triangle_number</t>
         </is>
       </c>
-      <c r="D2" t="n">
-        <v>1</v>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>largest_eigenvalue</t>
+        </is>
       </c>
       <c r="E2" t="n">
-        <v>12</v>
+        <v>128</v>
       </c>
       <c r="F2" t="n">
-        <v>20</v>
+        <v>9.277508673110397</v>
       </c>
       <c r="G2" t="n">
-        <v>4</v>
+        <v>0.05689384402057485</v>
       </c>
       <c r="H2" t="n">
-        <v>11</v>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>&gt;&gt;graph6&lt;&lt;KgDfH?@EGB?N</t>
-        </is>
+        <v>14</v>
+      </c>
+      <c r="I2" t="n">
+        <v>63</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>MvH^nf~~^RtnNlT__</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>search</t>
+        </is>
+      </c>
+      <c r="L2" t="n">
+        <v>102</v>
+      </c>
+      <c r="M2" t="n">
+        <v>1.797195672988892</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>980</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>average_degree</t>
-        </is>
+        <v>6472</v>
+      </c>
+      <c r="B3" t="b">
+        <v>1</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>clique_number</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>0.2142857142857144</v>
+          <t>triangle_number</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>largest_eigenvalue</t>
+        </is>
       </c>
       <c r="E3" t="n">
-        <v>14</v>
+        <v>100</v>
       </c>
       <c r="F3" t="n">
-        <v>16</v>
+        <v>8.53043406702392</v>
       </c>
       <c r="G3" t="n">
-        <v>2.285714285714286</v>
+        <v>0.002285998630629393</v>
       </c>
       <c r="H3" t="n">
-        <v>4</v>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>&gt;&gt;graph6&lt;&lt;MC??@?`MY??b?G?a?</t>
-        </is>
+        <v>13</v>
+      </c>
+      <c r="I3" t="n">
+        <v>54</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Lbp}x|vvf^U~qe</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>search</t>
+        </is>
+      </c>
+      <c r="L3" t="n">
+        <v>89</v>
+      </c>
+      <c r="M3" t="n">
+        <v>1.337033987045288</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>981</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>average_degree</t>
-        </is>
+        <v>7565</v>
+      </c>
+      <c r="B4" t="b">
+        <v>1</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>clique_number</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>0.1282051282051286</v>
+          <t>largest_eigenvalue</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>triangle_number</t>
+        </is>
       </c>
       <c r="E4" t="n">
-        <v>13</v>
+        <v>8.854330279962458</v>
       </c>
       <c r="F4" t="n">
-        <v>19</v>
+        <v>112</v>
       </c>
       <c r="G4" t="n">
-        <v>2.923076923076923</v>
+        <v>0.5794380998845554</v>
       </c>
       <c r="H4" t="n">
-        <v>5</v>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>&gt;&gt;graph6&lt;&lt;L@GG@T?IoBTI@?</t>
-        </is>
+        <v>11</v>
+      </c>
+      <c r="I4" t="n">
+        <v>46</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Jz~~~~~~{_?</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>search</t>
+        </is>
+      </c>
+      <c r="L4" t="n">
+        <v>84</v>
+      </c>
+      <c r="M4" t="n">
+        <v>1.350342273712158</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>1177</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>clique_number</t>
-        </is>
+        <v>7566</v>
+      </c>
+      <c r="B5" t="b">
+        <v>1</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>average_degree</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>0.06666666666666643</v>
+          <t>largest_eigenvalue</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>triangle_number</t>
+        </is>
       </c>
       <c r="E5" t="n">
-        <v>12</v>
+        <v>8.665141306429588</v>
       </c>
       <c r="F5" t="n">
-        <v>14</v>
+        <v>105</v>
       </c>
       <c r="G5" t="n">
-        <v>4</v>
+        <v>0.6746208428870943</v>
       </c>
       <c r="H5" t="n">
-        <v>2.333333333333333</v>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>&gt;&gt;graph6&lt;&lt;K?Ca??K_oS_R</t>
-        </is>
+        <v>11</v>
+      </c>
+      <c r="I5" t="n">
+        <v>45</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>J~~~~vn~wH?</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>search</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
+        <v>87</v>
+      </c>
+      <c r="M5" t="n">
+        <v>1.476248502731323</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>1178</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>clique_number</t>
-        </is>
+        <v>7811</v>
+      </c>
+      <c r="B6" t="b">
+        <v>1</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>average_degree</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>0.07692307692307709</v>
+          <t>second_smallest_laplace_eigenvalue</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>largest_eigenvalue</t>
+        </is>
       </c>
       <c r="E6" t="n">
-        <v>13</v>
+        <v>14.16563735746464</v>
       </c>
       <c r="F6" t="n">
-        <v>19</v>
+        <v>21.70330576626345</v>
       </c>
       <c r="G6" t="n">
-        <v>5</v>
+        <v>0.0885441855092246</v>
       </c>
       <c r="H6" t="n">
-        <v>2.923076923076923</v>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>&gt;&gt;graph6&lt;&lt;LJ]??GAO@C^O?O</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>1191</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>clique_number</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>minimum_degree</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>0.3350548340548301</v>
-      </c>
-      <c r="E7" t="n">
-        <v>13</v>
-      </c>
-      <c r="F7" t="n">
-        <v>67</v>
-      </c>
-      <c r="G7" t="n">
-        <v>8</v>
-      </c>
-      <c r="H7" t="n">
-        <v>9</v>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>&gt;&gt;graph6&lt;&lt;L~}^~~~~vZr^Nz</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>1466</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>domination_number</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>independent_domination_number</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>0.4867142857142959</v>
-      </c>
-      <c r="E8" t="n">
-        <v>14</v>
-      </c>
-      <c r="F8" t="n">
-        <v>16</v>
-      </c>
-      <c r="G8" t="n">
-        <v>5</v>
-      </c>
-      <c r="H8" t="n">
-        <v>6</v>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>&gt;&gt;graph6&lt;&lt;M@c?QK?COG@_CgC??</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>1566</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>total_domination_number</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>independence_number</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>1</v>
-      </c>
-      <c r="E9" t="n">
-        <v>10</v>
-      </c>
-      <c r="F9" t="n">
-        <v>12</v>
-      </c>
-      <c r="G9" t="n">
-        <v>6</v>
-      </c>
-      <c r="H9" t="n">
-        <v>4</v>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>&gt;&gt;graph6&lt;&lt;IgWO@Dk_?</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>1587</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>total_domination_number</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>matching_number</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>-1.666666666666668</v>
-      </c>
-      <c r="E10" t="n">
-        <v>24</v>
-      </c>
-      <c r="F10" t="n">
-        <v>23</v>
-      </c>
-      <c r="G10" t="n">
-        <v>13</v>
-      </c>
-      <c r="H10" t="n">
-        <v>10</v>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>&gt;&gt;graph6&lt;&lt;WhCGGC@?G?_@?@??o?@????CG??C??@???G????G?C????@</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>1588</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>total_domination_number</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>matching_number</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E11" t="n">
-        <v>15</v>
-      </c>
-      <c r="F11" t="n">
-        <v>14</v>
-      </c>
-      <c r="G11" t="n">
-        <v>8</v>
-      </c>
-      <c r="H11" t="n">
-        <v>5</v>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>&gt;&gt;graph6&lt;&lt;NC??J?@aDC?@@?C??_?</t>
-        </is>
+        <v>27</v>
+      </c>
+      <c r="I6" t="n">
+        <v>290</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Z~~}~~~~}~~nvy~v~}~u^z|~~vn}~q^s~zz~}t~n~yvgvpl~N~nwv^~atuww</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>search</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
+        <v>102</v>
+      </c>
+      <c r="M6" t="n">
+        <v>2.037301301956177</v>
       </c>
     </row>
   </sheetData>

</xml_diff>